<commit_message>
updated date in sources sheet
</commit_message>
<xml_diff>
--- a/Collected Studies.xlsx
+++ b/Collected Studies.xlsx
@@ -1567,7 +1567,7 @@
     <t>The effect of risk assessment scores on judicial behavior and defendant outcomes</t>
   </si>
   <si>
-    <t>Sloan, CarlyWill, George Naufal, and Heather Caspers</t>
+    <t>Sloan, Carly Will, George Naufal, and Heather Caspers</t>
   </si>
   <si>
     <t>Journal of Human Resources</t>
@@ -5591,7 +5591,7 @@
         <v>516</v>
       </c>
       <c r="D45" s="3">
-        <v>2020.0</v>
+        <v>2025.0</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>517</v>
@@ -65125,7 +65125,7 @@
       </c>
       <c r="G7" s="11">
         <f>COUNTIF(Included!$D:$D, "=2020")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H7" s="11">
         <f>COUNTIF(Included!$D:$D, "=2021")</f>
@@ -65145,7 +65145,7 @@
       </c>
       <c r="L7" s="11">
         <f>COUNTIF(Included!$D:$D, "=2025")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="11">
         <f>COUNTIF(Included!$D:$D, "=2026")</f>

</xml_diff>